<commit_message>
feat: iniciar fundacao web do Expert para CompreMai Estivas
</commit_message>
<xml_diff>
--- a/docs/escopo_erp_pdv_web_revisado.xlsx
+++ b/docs/escopo_erp_pdv_web_revisado.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="R714806ac75604850"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stack Tecnológica" sheetId="2" r:id="R3e53951fae4c4f9c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Módulos" sheetId="3" r:id="Rec488efbaf264f87"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relatórios" sheetId="4" r:id="Rf12b9db7e3c147a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fiscal e Roadmap" sheetId="5" r:id="Rfbaa73611ebd419c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lacunas e decisões" sheetId="6" r:id="Rd3d98ce7a0534e62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="Rc8f7d5ac66a74dcb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stack Tecnológica" sheetId="2" r:id="R5422db8cb7e64cce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Módulos" sheetId="3" r:id="R3ec8d5a32edf4091"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relatórios" sheetId="4" r:id="R9f50ace4f4cb442a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fiscal e Roadmap" sheetId="5" r:id="R814eb202ad7d4db8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lacunas e decisões" sheetId="6" r:id="Rfdb8d0e1276c4069"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -506,7 +506,7 @@
     </x:row>
     <x:row r="2" ht="27" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>Projeto do zero • painel e PDV no navegador • emissão fiscal no servidor • revisão em 16/09/2026</x:v>
+        <x:v>CompreMai$ Estivas • varejo supermercadista no RN • painel e PDV web • revisão em 16/09/2026</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -878,13 +878,13 @@
     </x:row>
     <x:row r="23" ht="49" customHeight="1">
       <x:c r="A23" s="12" t="str">
-        <x:v>Piloto recomendado</x:v>
+        <x:v>Piloto CompreMai$ Estivas</x:v>
       </x:c>
       <x:c r="B23" s="12" t="str">
         <x:v>Uma loja</x:v>
       </x:c>
       <x:c r="C23" s="12" t="str">
-        <x:v>Uma UF</x:v>
+        <x:v>RN</x:v>
       </x:c>
       <x:c r="D23" s="12" t="str">
         <x:v>HTTPS</x:v>
@@ -1565,7 +1565,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc9e04897e47c45d4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a6d6f29b660436d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1596,7 +1596,7 @@
     </x:row>
     <x:row r="2" ht="27" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>Proposta de MVP em uma loja e uma UF. Produtos concretos serão definidos após o escopo.</x:v>
+        <x:v>Piloto CompreMai$ Estivas: varejo supermercadista no RN. Produtos reais serão definidos com a loja.</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -2610,7 +2610,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfbd2ec097994423e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc490f93fe49e4596"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3065,8 +3065,8 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd9b448d9e4d0485b"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac7196d2a8714369"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf70f496edf64ea0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdff5b56964614682"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3854,7 +3854,7 @@
         <x:v>Escopo fechado</x:v>
       </x:c>
       <x:c r="D36" s="15" t="str">
-        <x:v>Varejo, uma loja/UF, fluxos e matriz fiscal; produtos detalhados depois</x:v>
+        <x:v>CompreMai$ Estivas, supermercado no RN; fluxos e matriz fiscal; produtos reais depois</x:v>
       </x:c>
       <x:c r="E36" s="15" t="str">
         <x:v>Backlog, protótipo e decisões registradas</x:v>
@@ -4153,9 +4153,9 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="3">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4dfa9fbc6b2747bc"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5a55e7dce50d4682"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0303676493754cd9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R82d19e38884b435a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R08dadb3673044da0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77f9f0c738a546bf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4232,13 +4232,13 @@
         <x:v>Segmento</x:v>
       </x:c>
       <x:c r="B5" s="12" t="str">
-        <x:v>Cliente e operação alvo não definidos</x:v>
+        <x:v>CompreMai$ Estivas informado como piloto</x:v>
       </x:c>
       <x:c r="C5" s="12" t="str">
-        <x:v>Piloto em varejo de mercadorias; serviços em fase posterior</x:v>
+        <x:v>Varejo supermercadista para uma loja inicial</x:v>
       </x:c>
       <x:c r="D5" s="12" t="str">
-        <x:v>Processos de uma loja descritos e aprovados</x:v>
+        <x:v>Processos reais da loja descritos e aprovados</x:v>
       </x:c>
       <x:c r="E5" s="12" t="str">
         <x:v>Empresário</x:v>
@@ -4247,7 +4247,7 @@
         <x:v>Crítica</x:v>
       </x:c>
       <x:c r="G5" s="12" t="str">
-        <x:v>Pendente</x:v>
+        <x:v>Resolvido</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="62" customHeight="1">
@@ -4255,10 +4255,10 @@
         <x:v>UF e regime</x:v>
       </x:c>
       <x:c r="B6" s="15" t="str">
-        <x:v>Não há UF nem regime tributário piloto</x:v>
+        <x:v>RN definido; regime tributário e contador pendentes</x:v>
       </x:c>
       <x:c r="C6" s="15" t="str">
-        <x:v>Escolher uma UF, regime e contador antes do fiscal</x:v>
+        <x:v>Fechar regime e matriz fiscal do RN antes da emissão</x:v>
       </x:c>
       <x:c r="D6" s="15" t="str">
         <x:v>Matriz fiscal e credenciamento confirmados</x:v>
@@ -4270,7 +4270,7 @@
         <x:v>Crítica</x:v>
       </x:c>
       <x:c r="G6" s="15" t="str">
-        <x:v>Pendente</x:v>
+        <x:v>Em validação</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="62" customHeight="1">
@@ -4730,7 +4730,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf43390fcc0643cf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R819f31d6dc474fad"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: preparar fechamento de caixa e finalizadoras do PDV
</commit_message>
<xml_diff>
--- a/docs/escopo_erp_pdv_web_revisado.xlsx
+++ b/docs/escopo_erp_pdv_web_revisado.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="Rc8f7d5ac66a74dcb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stack Tecnológica" sheetId="2" r:id="R5422db8cb7e64cce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Módulos" sheetId="3" r:id="R3ec8d5a32edf4091"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relatórios" sheetId="4" r:id="R9f50ace4f4cb442a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fiscal e Roadmap" sheetId="5" r:id="R814eb202ad7d4db8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lacunas e decisões" sheetId="6" r:id="Rfdb8d0e1276c4069"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="R54bd5fd92cb44e86"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stack Tecnológica" sheetId="2" r:id="Rb61a0b0a1bff4407"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Módulos" sheetId="3" r:id="Rd49ed34cad1d4161"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relatórios" sheetId="4" r:id="R7b4e22afd07f48f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fiscal e Roadmap" sheetId="5" r:id="Rf37ebcc697834ec4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lacunas e decisões" sheetId="6" r:id="R1a12a81513de49fd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -173,8 +173,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ModulosERP" displayName="ModulosERP" ref="A4:G46" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:G46"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ModulosERP" displayName="ModulosERP" ref="A4:G50" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:G50"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="Domínio"/>
     <x:tableColumn id="2" name="Módulo"/>
@@ -189,8 +189,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="CatalogoRelatorios" displayName="CatalogoRelatorios" ref="A4:G9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A4:G9"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="CatalogoRelatorios" displayName="CatalogoRelatorios" ref="A4:G10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:G10"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="Relatório"/>
     <x:tableColumn id="2" name="Visão"/>
@@ -205,8 +205,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="RegrasRelatorios" displayName="RegrasRelatorios" ref="A12:G20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A12:G20"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="RegrasRelatorios" displayName="RegrasRelatorios" ref="A12:G21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A12:G21"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="Regra"/>
     <x:tableColumn id="2" name="Definição"/>
@@ -1565,7 +1565,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a6d6f29b660436d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d8cdd2e880c41b3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2603,6 +2603,98 @@
         <x:v>Alta</x:v>
       </x:c>
     </x:row>
+    <x:row r="47" ht="55" customHeight="1">
+      <x:c r="A47" s="12" t="str">
+        <x:v>PDV</x:v>
+      </x:c>
+      <x:c r="B47" s="12" t="str">
+        <x:v>Conferência e fechamento de caixa</x:v>
+      </x:c>
+      <x:c r="C47" s="12" t="str">
+        <x:v>Abertura, suprimentos, sangrias, pagamentos, estornos e conferência por meio, inclusive Convênio e Troca</x:v>
+      </x:c>
+      <x:c r="D47" s="12" t="str">
+        <x:v>Sim</x:v>
+      </x:c>
+      <x:c r="E47" s="12" t="str">
+        <x:v>Sessão / venda / pagamentos</x:v>
+      </x:c>
+      <x:c r="F47" s="12" t="str">
+        <x:v>Previsto, conferido e diferença por meio; observação e trilha do operador</x:v>
+      </x:c>
+      <x:c r="G47" s="12" t="str">
+        <x:v>Crítica</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="55" customHeight="1">
+      <x:c r="A48" s="15" t="str">
+        <x:v>Relatórios</x:v>
+      </x:c>
+      <x:c r="B48" s="15" t="str">
+        <x:v>Fechamento dos PDVs</x:v>
+      </x:c>
+      <x:c r="C48" s="15" t="str">
+        <x:v>Comprovante não fiscal no caixa e consulta consolidada na retaguarda</x:v>
+      </x:c>
+      <x:c r="D48" s="15" t="str">
+        <x:v>Sim</x:v>
+      </x:c>
+      <x:c r="E48" s="15" t="str">
+        <x:v>Sessão / check-out / usuário</x:v>
+      </x:c>
+      <x:c r="F48" s="15" t="str">
+        <x:v>Filtro por período, filial, caixa e operador; reimpressão vinculada ao fechamento</x:v>
+      </x:c>
+      <x:c r="G48" s="15" t="str">
+        <x:v>Alta</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="55" customHeight="1">
+      <x:c r="A49" s="12" t="str">
+        <x:v>PDV</x:v>
+      </x:c>
+      <x:c r="B49" s="12" t="str">
+        <x:v>Integração TEF</x:v>
+      </x:c>
+      <x:c r="C49" s="12" t="str">
+        <x:v>Aprovação, consulta de transação incerta, cancelamento, estorno, comprovantes e conciliação</x:v>
+      </x:c>
+      <x:c r="D49" s="12" t="str">
+        <x:v>Sim</x:v>
+      </x:c>
+      <x:c r="E49" s="12" t="str">
+        <x:v>Provedor a definir / terminal</x:v>
+      </x:c>
+      <x:c r="F49" s="12" t="str">
+        <x:v>Venda não conclui sem pagamento confirmado; timeout não duplica cobrança</x:v>
+      </x:c>
+      <x:c r="G49" s="12" t="str">
+        <x:v>Crítica</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="55" customHeight="1">
+      <x:c r="A50" s="15" t="str">
+        <x:v>PDV</x:v>
+      </x:c>
+      <x:c r="B50" s="15" t="str">
+        <x:v>Finalizadoras Convênio e Troca</x:v>
+      </x:c>
+      <x:c r="C50" s="15" t="str">
+        <x:v>Convênio vinculado a conveniado e contas a receber; Troca consome crédito de devolução rastreável</x:v>
+      </x:c>
+      <x:c r="D50" s="15" t="str">
+        <x:v>Sim</x:v>
+      </x:c>
+      <x:c r="E50" s="15" t="str">
+        <x:v>Clientes / devoluções / financeiro</x:v>
+      </x:c>
+      <x:c r="F50" s="15" t="str">
+        <x:v>Autorização, limite e saldo validados; sem dupla contagem de faturamento</x:v>
+      </x:c>
+      <x:c r="G50" s="15" t="str">
+        <x:v>Alta</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:G1"/>
@@ -2610,7 +2702,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc490f93fe49e4596"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f99182026d34cc7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2797,14 +2889,28 @@
         <x:v>2. PDV</x:v>
       </x:c>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="2"/>
-      <x:c r="B10" s="2"/>
-      <x:c r="C10" s="2"/>
-      <x:c r="D10" s="2"/>
-      <x:c r="E10" s="2"/>
-      <x:c r="F10" s="2"/>
-      <x:c r="G10" s="2"/>
+    <x:row r="10" ht="91" customHeight="1">
+      <x:c r="A10" s="15" t="str">
+        <x:v>Fechamento dos PDVs</x:v>
+      </x:c>
+      <x:c r="B10" s="15" t="str">
+        <x:v>Turno e check-out; comprovante individual e resumo da retaguarda</x:v>
+      </x:c>
+      <x:c r="C10" s="15" t="str">
+        <x:v>Data/hora do fechamento no fuso da filial</x:v>
+      </x:c>
+      <x:c r="D10" s="15" t="str">
+        <x:v>Filial, check-out, operador, período, status, divergência</x:v>
+      </x:c>
+      <x:c r="E10" s="15" t="str">
+        <x:v>Fundo, suprimento, sangria, venda e estorno; previsto, conferido e diferença por meio, inclusive Convênio e Troca</x:v>
+      </x:c>
+      <x:c r="F10" s="15" t="str">
+        <x:v>Dinheiro inclui fundo e movimentos; vendas líquidas à parte; trilha e reimpressão</x:v>
+      </x:c>
+      <x:c r="G10" s="15" t="str">
+        <x:v>2. PDV</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="25" customHeight="1">
       <x:c r="A11" s="8" t="str">
@@ -3024,14 +3130,28 @@
         <x:v>Registrar exportações</x:v>
       </x:c>
     </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="2"/>
-      <x:c r="B21" s="2"/>
-      <x:c r="C21" s="2"/>
-      <x:c r="D21" s="2"/>
-      <x:c r="E21" s="2"/>
-      <x:c r="F21" s="2"/>
-      <x:c r="G21" s="2"/>
+    <x:row r="21" ht="65" customHeight="1">
+      <x:c r="A21" s="12" t="str">
+        <x:v>Fechamento</x:v>
+      </x:c>
+      <x:c r="B21" s="12" t="str">
+        <x:v>Diferença = conferido - previsto por meio; dinheiro inclui fundo + vendas + suprimentos - sangrias - estornos</x:v>
+      </x:c>
+      <x:c r="C21" s="12" t="str">
+        <x:v>Total confere com soma das linhas; divergência exige observação e responsável</x:v>
+      </x:c>
+      <x:c r="D21" s="12" t="str">
+        <x:v>Sessão, pagamentos e movimentos</x:v>
+      </x:c>
+      <x:c r="E21" s="12" t="str">
+        <x:v>Operação + TI</x:v>
+      </x:c>
+      <x:c r="F21" s="12" t="str">
+        <x:v>Definido</x:v>
+      </x:c>
+      <x:c r="G21" s="12" t="str">
+        <x:v>Comprovante não fiscal; Elgin i9, i9 Full e i9 Full2 a homologar</x:v>
+      </x:c>
     </x:row>
     <x:row r="22" ht="25" customHeight="1">
       <x:c r="A22" s="8" t="str">
@@ -3046,7 +3166,7 @@
     </x:row>
     <x:row r="23" ht="44" customHeight="1">
       <x:c r="A23" s="17" t="str">
-        <x:v>Cadastro de produtos na fundação; PDV por check-out na fase 2; vendas fiscais na fase 3; entradas de mercadorias após compras e recebimento na fase 6.</x:v>
+        <x:v>Cadastro de produtos na fundação; vendas e fechamento dos PDVs na fase 2; vendas fiscais na fase 3; entradas de mercadorias após compras e recebimento na fase 6.</x:v>
       </x:c>
       <x:c r="B23" s="17"/>
       <x:c r="C23" s="17"/>
@@ -3065,8 +3185,8 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf70f496edf64ea0"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdff5b56964614682"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R33a397c5ca244281"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R382d5201d7574b5f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3906,10 +4026,10 @@
         <x:v>Venda operacional</x:v>
       </x:c>
       <x:c r="D38" s="15" t="str">
-        <x:v>Preço, caixa, pagamento, estoque, devolução e relatório por check-out</x:v>
+        <x:v>Preço, caixa, TEF, Convênio, Troca, estoque, devolução, fechamento e relatórios por check-out</x:v>
       </x:c>
       <x:c r="E38" s="15" t="str">
-        <x:v>Venda, estoque, caixa e ticket médio conciliam</x:v>
+        <x:v>Venda, estoque, caixa, ticket médio e fechamento conciliam</x:v>
       </x:c>
       <x:c r="F38" s="15" t="str">
         <x:v>Inconsistência transacional</x:v>
@@ -4153,9 +4273,9 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="3">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R82d19e38884b435a"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R08dadb3673044da0"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77f9f0c738a546bf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb64b421b23454789"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda9f5907efbb45e3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ad699000b5646f5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4347,13 +4467,13 @@
         <x:v>Periféricos</x:v>
       </x:c>
       <x:c r="B10" s="15" t="str">
-        <x:v>Impressão, balança e gaveta sem matriz de suporte</x:v>
+        <x:v>Elgin i9, i9 Full e i9 Full2 indicadas; navegador e SO pendentes</x:v>
       </x:c>
       <x:c r="C10" s="15" t="str">
-        <x:v>Homologar SO, navegador e modelos reais; usar print do browser</x:v>
+        <x:v>Testar bobina, margens, corte e diálogo de impressão nos três modelos</x:v>
       </x:c>
       <x:c r="D10" s="15" t="str">
-        <x:v>Roteiro no caixa real e plano de falha</x:v>
+        <x:v>Comprovante legível em cada caixa real e plano de falha</x:v>
       </x:c>
       <x:c r="E10" s="15" t="str">
         <x:v>Operação + TI</x:v>
@@ -4362,7 +4482,7 @@
         <x:v>Crítica</x:v>
       </x:c>
       <x:c r="G10" s="15" t="str">
-        <x:v>Pendente</x:v>
+        <x:v>Em validação</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="62" customHeight="1">
@@ -4370,22 +4490,22 @@
         <x:v>Pagamentos</x:v>
       </x:c>
       <x:c r="B11" s="12" t="str">
-        <x:v>Cartão/PIX registrados sem retorno transacional</x:v>
+        <x:v>Provedor TEF a definir; regras de Convênio e Troca pendentes</x:v>
       </x:c>
       <x:c r="C11" s="12" t="str">
-        <x:v>MVP registra comprovante; TEF/API após contrato e integração</x:v>
+        <x:v>Escolher integração e mapear autorização, limite, crédito e conciliação</x:v>
       </x:c>
       <x:c r="D11" s="12" t="str">
-        <x:v>Conciliação sem pagamento fantasma</x:v>
+        <x:v>Pagamento confirmado sem duplicidade e crédito rastreável</x:v>
       </x:c>
       <x:c r="E11" s="12" t="str">
         <x:v>Empresa + TI</x:v>
       </x:c>
       <x:c r="F11" s="12" t="str">
-        <x:v>Alta</x:v>
+        <x:v>Crítica</x:v>
       </x:c>
       <x:c r="G11" s="12" t="str">
-        <x:v>Pendente</x:v>
+        <x:v>Em validação</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="62" customHeight="1">
@@ -4730,7 +4850,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R819f31d6dc474fad"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe427e8b343f4e82"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
docs: atualizar data da revisao do escopo
</commit_message>
<xml_diff>
--- a/docs/escopo_erp_pdv_web_revisado.xlsx
+++ b/docs/escopo_erp_pdv_web_revisado.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="R54bd5fd92cb44e86"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stack Tecnológica" sheetId="2" r:id="Rb61a0b0a1bff4407"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Módulos" sheetId="3" r:id="Rd49ed34cad1d4161"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relatórios" sheetId="4" r:id="R7b4e22afd07f48f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fiscal e Roadmap" sheetId="5" r:id="Rf37ebcc697834ec4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lacunas e decisões" sheetId="6" r:id="R1a12a81513de49fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumo" sheetId="1" r:id="R90abe01500654427"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stack Tecnológica" sheetId="2" r:id="R59b42e4c4143472c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Módulos" sheetId="3" r:id="R8324b850b8d6409f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relatórios" sheetId="4" r:id="Rfc974bb648854eff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fiscal e Roadmap" sheetId="5" r:id="Ra84b48216f4f4f81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lacunas e decisões" sheetId="6" r:id="R48b1d4c0cadf4bdb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -506,7 +506,7 @@
     </x:row>
     <x:row r="2" ht="27" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>CompreMai$ Estivas • varejo supermercadista no RN • painel e PDV web • revisão em 16/09/2026</x:v>
+        <x:v>CompreMai$ Estivas • varejo supermercadista no RN • painel e PDV web • revisão em 17/09/2026</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -1565,7 +1565,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6d8cdd2e880c41b3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R049c1fc697974bcf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2702,7 +2702,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f99182026d34cc7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R91a8fda55cda4155"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3185,8 +3185,8 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R33a397c5ca244281"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R382d5201d7574b5f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R27f1de0e0dfc4529"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0d26433f53e145bf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4273,9 +4273,9 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="3">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb64b421b23454789"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda9f5907efbb45e3"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ad699000b5646f5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Refc2b3022f594de6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37f08f383d7c4a12"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R598dc56685974735"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4850,7 +4850,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe427e8b343f4e82"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5402b2560db94bb9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>